<commit_message>
docs: add AI audit log and project presentation slides
</commit_message>
<xml_diff>
--- a/Documents/AI_AuditLog_26SU_SE20B02_G1_IOT102.xlsx
+++ b/Documents/AI_AuditLog_26SU_SE20B02_G1_IOT102.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Officefiles\Ki_4\IOT102\KidCheck-IOT102\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{671E42B8-7456-48C1-A91B-DE0802633DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2758DE2A-ECE4-4663-B9F3-74D882DB4FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1063,12 +1063,12 @@
     <col min="1" max="1" width="8" style="1" customWidth="1"/>
     <col min="2" max="2" width="18" style="1" customWidth="1"/>
     <col min="3" max="3" width="20" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" style="1" customWidth="1"/>
     <col min="5" max="5" width="20" style="1" customWidth="1"/>
     <col min="6" max="6" width="30" style="1" customWidth="1"/>
     <col min="7" max="7" width="45" style="1" customWidth="1"/>
     <col min="8" max="9" width="40" style="1" customWidth="1"/>
-    <col min="10" max="10" width="20" style="1" customWidth="1"/>
+    <col min="10" max="10" width="29.42578125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -1487,7 +1487,7 @@
         <v>95</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>28</v>
+        <v>199</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>96</v>

</xml_diff>